<commit_message>
Mejoras en formato revaluacion de proveedores: uso de fecha de aprobacion en lugar de suscripcion, conversion de adicion a letras de manera automatica y ordenamiento por numero de contrato en tabla.
</commit_message>
<xml_diff>
--- a/plantillas/REVALUACION_PROVEEDORES_TEMPLATE.xlsx
+++ b/plantillas/REVALUACION_PROVEEDORES_TEMPLATE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soporte y Desarrollo\Documents\NetBeansProjects\combinacion\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AAA1580-3B95-4DBC-B44E-8EA902A35950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D822727D-76D2-4676-96C0-BC5A86486021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -304,13 +304,13 @@
     </r>
   </si>
   <si>
-    <t>${DIA_SUSC}</t>
-  </si>
-  <si>
-    <t>${MES_SUSC}</t>
-  </si>
-  <si>
-    <t>${ANIO_SUSC}</t>
+    <t>${DIA_APROBACION}</t>
+  </si>
+  <si>
+    <t>${MES_APROBACION}</t>
+  </si>
+  <si>
+    <t>${ANIO_APROBACION}</t>
   </si>
 </sst>
 </file>

</xml_diff>